<commit_message>
chore: update MPFA open data
</commit_message>
<xml_diff>
--- a/data/current/number-of-mpf-intermediaries/en/number_of_mpf_intermediaries01_en.xlsx
+++ b/data/current/number-of-mpf-intermediaries/en/number_of_mpf_intermediaries01_en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\oaserv01\Research\Statistics &amp; Research\Statistics Report\04 Monthly\PSI Portal\2026\202608\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\oaserv01\Research\Statistics &amp; Research\Statistics Report\04 Monthly\PSI Portal\2026\202609\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696834C0-7F9A-4542-B5BD-0BCA8810429F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A3A9AB-B19B-474A-9BEC-E88BEDA16D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>As at</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>31-08-2026</t>
+  </si>
+  <si>
+    <t>30-09-2026</t>
   </si>
 </sst>
 </file>
@@ -688,7 +691,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -1586,6 +1589,17 @@
         <v>40714</v>
       </c>
     </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B82" s="4">
+        <v>433</v>
+      </c>
+      <c r="C82" s="4">
+        <v>40960</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>